<commit_message>
Updated machine IP Addresses
git-svn-id: http://10.105.1.46/svn/CCRT/Ccrt/branches/Common3700@16713 80089e14-fa6c-c64e-badd-1f0333e23b03
</commit_message>
<xml_diff>
--- a/Source/Mazda/Mazda Plant Matrix.xlsx
+++ b/Source/Mazda/Mazda Plant Matrix.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="1635" yWindow="1650" windowWidth="27795" windowHeight="12525"/>
+    <workbookView xWindow="-420" yWindow="3120" windowWidth="27795" windowHeight="12525"/>
   </bookViews>
   <sheets>
     <sheet name="Salamanca" sheetId="8" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="51">
   <si>
     <t>S / N</t>
   </si>
@@ -135,13 +135,40 @@
     <t>Side Slip</t>
   </si>
   <si>
-    <t>192.168.1.1</t>
-  </si>
-  <si>
-    <t>192.168.3.1</t>
-  </si>
-  <si>
     <t>192.168.2.1</t>
+  </si>
+  <si>
+    <t>Brake Tester</t>
+  </si>
+  <si>
+    <t>7 - Home</t>
+  </si>
+  <si>
+    <t>6.3.2</t>
+  </si>
+  <si>
+    <t>10.236.87.61</t>
+  </si>
+  <si>
+    <t>10.236.87.60</t>
+  </si>
+  <si>
+    <t>Mazda</t>
+  </si>
+  <si>
+    <t>BrakeTest</t>
+  </si>
+  <si>
+    <t>Roll Tester</t>
+  </si>
+  <si>
+    <t>10.236.87.76</t>
+  </si>
+  <si>
+    <t>10.236.87.75</t>
+  </si>
+  <si>
+    <t>RollTest</t>
   </si>
 </sst>
 </file>
@@ -159,6 +186,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -395,7 +423,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -484,6 +512,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -799,7 +833,7 @@
     <col min="6" max="6" width="24.42578125" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.42578125" customWidth="1"/>
     <col min="12" max="12" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18.42578125" bestFit="1" customWidth="1"/>
@@ -973,39 +1007,75 @@
       </c>
     </row>
     <row r="19" spans="1:15" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="17"/>
-      <c r="B19" s="31"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5" t="s">
-        <v>39</v>
+      <c r="A19" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="31">
+        <v>507769</v>
+      </c>
+      <c r="C19" s="31">
+        <v>3700</v>
+      </c>
+      <c r="D19" s="39" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="39" t="s">
+        <v>42</v>
+      </c>
+      <c r="F19" s="39" t="s">
+        <v>43</v>
       </c>
       <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
+      <c r="H19" s="5" t="s">
+        <v>44</v>
+      </c>
       <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
+      <c r="J19" s="39" t="s">
+        <v>45</v>
+      </c>
+      <c r="K19" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="L19" s="5">
+        <v>1</v>
+      </c>
       <c r="M19" s="5"/>
       <c r="N19" s="18"/>
       <c r="O19" s="24"/>
     </row>
     <row r="20" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="14"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
+      <c r="A20" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" s="5">
+        <v>507768</v>
+      </c>
+      <c r="C20" s="5">
+        <v>3700</v>
+      </c>
+      <c r="D20" s="39" t="s">
+        <v>41</v>
+      </c>
+      <c r="E20" s="39" t="s">
+        <v>42</v>
+      </c>
       <c r="F20" s="5" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
+      <c r="H20" s="5" t="s">
+        <v>49</v>
+      </c>
       <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
+      <c r="J20" s="39" t="s">
+        <v>45</v>
+      </c>
+      <c r="K20" s="39" t="s">
+        <v>50</v>
+      </c>
+      <c r="L20" s="5">
+        <v>1</v>
+      </c>
       <c r="M20" s="5"/>
       <c r="N20" s="18"/>
       <c r="O20" s="24"/>
@@ -1214,7 +1284,7 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F33" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added new line machines.
git-svn-id: http://10.105.1.46/svn/CCRT/Ccrt/branches/Common3700@16957 80089e14-fa6c-c64e-badd-1f0333e23b03
</commit_message>
<xml_diff>
--- a/Source/Mazda/Mazda Plant Matrix.xlsx
+++ b/Source/Mazda/Mazda Plant Matrix.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="55">
   <si>
     <t>S / N</t>
   </si>
@@ -169,6 +169,18 @@
   </si>
   <si>
     <t>RollTest</t>
+  </si>
+  <si>
+    <t>192.168.1.1</t>
+  </si>
+  <si>
+    <t>192.168.1.2</t>
+  </si>
+  <si>
+    <t>192.168.3.1</t>
+  </si>
+  <si>
+    <t>192.168.3.2</t>
   </si>
 </sst>
 </file>
@@ -423,7 +435,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -518,6 +530,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1098,35 +1113,71 @@
       <c r="O21" s="24"/>
     </row>
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="16"/>
+      <c r="A22" s="40" t="s">
+        <v>40</v>
+      </c>
       <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
+      <c r="C22" s="5">
+        <v>3700</v>
+      </c>
+      <c r="D22" s="39" t="s">
+        <v>41</v>
+      </c>
+      <c r="E22" s="39" t="s">
+        <v>42</v>
+      </c>
+      <c r="F22" s="39" t="s">
+        <v>51</v>
+      </c>
       <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
+      <c r="H22" s="39" t="s">
+        <v>52</v>
+      </c>
       <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5"/>
+      <c r="J22" s="39" t="s">
+        <v>45</v>
+      </c>
+      <c r="K22" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="L22" s="5">
+        <v>2</v>
+      </c>
       <c r="M22" s="5"/>
       <c r="N22" s="18"/>
       <c r="O22" s="24"/>
     </row>
     <row r="23" spans="1:15" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="15"/>
+      <c r="A23" s="15" t="s">
+        <v>47</v>
+      </c>
       <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
+      <c r="C23" s="5">
+        <v>3700</v>
+      </c>
+      <c r="D23" s="39" t="s">
+        <v>41</v>
+      </c>
+      <c r="E23" s="39" t="s">
+        <v>42</v>
+      </c>
+      <c r="F23" s="39" t="s">
+        <v>53</v>
+      </c>
       <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
+      <c r="H23" s="39" t="s">
+        <v>54</v>
+      </c>
       <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
+      <c r="J23" s="39" t="s">
+        <v>45</v>
+      </c>
+      <c r="K23" s="39" t="s">
+        <v>50</v>
+      </c>
+      <c r="L23" s="5">
+        <v>2</v>
+      </c>
       <c r="M23" s="5"/>
       <c r="N23" s="18"/>
       <c r="O23" s="24"/>

</xml_diff>

<commit_message>
updated IP Addresses of lane 2 machines.
git-svn-id: http://10.105.1.46/svn/CCRT/Ccrt/branches/Common3700@17615 80089e14-fa6c-c64e-badd-1f0333e23b03
</commit_message>
<xml_diff>
--- a/Source/Mazda/Mazda Plant Matrix.xlsx
+++ b/Source/Mazda/Mazda Plant Matrix.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="-420" yWindow="3120" windowWidth="27795" windowHeight="12525"/>
@@ -171,16 +171,16 @@
     <t>RollTest</t>
   </si>
   <si>
-    <t>192.168.1.1</t>
-  </si>
-  <si>
-    <t>192.168.1.2</t>
-  </si>
-  <si>
-    <t>192.168.3.1</t>
-  </si>
-  <si>
-    <t>192.168.3.2</t>
+    <t>10.236.87.55</t>
+  </si>
+  <si>
+    <t>10.236.87.56</t>
+  </si>
+  <si>
+    <t>10.236.87.80</t>
+  </si>
+  <si>
+    <t>10.236.87.81</t>
   </si>
 </sst>
 </file>
@@ -435,7 +435,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -533,6 +533,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1127,11 +1130,11 @@
         <v>42</v>
       </c>
       <c r="F22" s="39" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G22" s="5"/>
       <c r="H22" s="39" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I22" s="5"/>
       <c r="J22" s="39" t="s">
@@ -1162,11 +1165,11 @@
         <v>42</v>
       </c>
       <c r="F23" s="39" t="s">
+        <v>54</v>
+      </c>
+      <c r="G23" s="5"/>
+      <c r="H23" s="41" t="s">
         <v>53</v>
-      </c>
-      <c r="G23" s="5"/>
-      <c r="H23" s="39" t="s">
-        <v>54</v>
       </c>
       <c r="I23" s="5"/>
       <c r="J23" s="39" t="s">

</xml_diff>

<commit_message>
Update to add new machines to the Mazda Plant Matrix.
git-svn-id: http://10.105.1.46/svn/CCRT/Ccrt/branches/Common3700@18315 80089e14-fa6c-c64e-badd-1f0333e23b03
</commit_message>
<xml_diff>
--- a/Source/Mazda/Mazda Plant Matrix.xlsx
+++ b/Source/Mazda/Mazda Plant Matrix.xlsx
@@ -1119,7 +1119,9 @@
       <c r="A22" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="5"/>
+      <c r="B22" s="5">
+        <v>508038</v>
+      </c>
       <c r="C22" s="5">
         <v>3700</v>
       </c>
@@ -1154,7 +1156,9 @@
       <c r="A23" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="5"/>
+      <c r="B23" s="5">
+        <v>508040</v>
+      </c>
       <c r="C23" s="5">
         <v>3700</v>
       </c>

</xml_diff>